<commit_message>
Dashboard v2: remove qualifying dates, add level ranks, disclaimer, refresh visuals
</commit_message>
<xml_diff>
--- a/docs/exports/area/Division_A_Area_01.xlsx
+++ b/docs/exports/area/Division_A_Area_01.xlsx
@@ -1,16 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Area 01 — Level Totals (Divi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Club Leaderboard (within Are" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pathways Quality Award — Exc" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pathways Quality Award — Sta" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Area 01 — Level Totals (Divi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="District-Wide Standing — Ran" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Club Leaderboard (within Are" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Pathways Quality Award — Exc" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Pathways Quality Award — Sta" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -579,6 +580,106 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>District 82 — Division A, Area 01 Director Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Pathways Education Performance — Area 01</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Snapshot as of 2026-06-30  |  District 82 Toastmasters Pathways Dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>District-Wide Standing — Rank Among All Areas</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Level 1 Rank</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Level 2 Rank</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Level 3 Rank</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Level 4+ Rank</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Total Levels Rank</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Out of 36 areas in the district.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -807,22 +908,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -876,15 +975,9 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Qualifying Date</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
           <t>Ovation 2027</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -900,30 +993,25 @@
       <c r="C7" s="6" t="inlineStr"/>
       <c r="D7" s="6" t="inlineStr"/>
       <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -975,13 +1063,6 @@
           <t>Level 3</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Qualifying Date</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr"/>
-      <c r="G6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
@@ -998,13 +1079,6 @@
       <c r="D7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -1021,13 +1095,6 @@
       <c r="D8" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr"/>
-      <c r="G8" s="8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
@@ -1044,13 +1111,6 @@
       <c r="D9" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr"/>
-      <c r="G9" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix rank consistency, remove Ovation mentions, declutter Areas tab, add report generated date
</commit_message>
<xml_diff>
--- a/docs/exports/area/Division_A_Area_01.xlsx
+++ b/docs/exports/area/Division_A_Area_01.xlsx
@@ -10,8 +10,8 @@
     <sheet name="Area 01 — Level Totals (Divi" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="District-Wide Standing — Ran" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Club Leaderboard (within Are" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Pathways Quality Award — Exc" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Pathways Quality Award — Sta" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Clubs Qualifying — Excellenc" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Clubs Qualifying — Star (thi" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -514,7 +514,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Snapshot as of 2026-06-30  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-30  |  Report generated 01 Jul 2026, 17:26  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Snapshot as of 2026-06-30  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-30  |  Report generated 01 Jul 2026, 17:26  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Snapshot as of 2026-06-30  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-30  |  Report generated 01 Jul 2026, 17:26  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -797,26 +797,26 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Lions Toastmasters Club</t>
+          <t>Commercial Bank Toastmasters Club</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E8" s="8" t="n">
         <v>2</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G8" s="8" t="n">
         <v>14</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>25</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9">
@@ -825,26 +825,26 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Commercial Bank Toastmasters Club</t>
+          <t>Lions Toastmasters Club</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" s="6" t="n">
         <v>4</v>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>6</v>
       </c>
       <c r="E9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G9" s="6" t="n">
         <v>14</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10">
@@ -914,14 +914,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -941,58 +939,42 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Snapshot as of 2026-06-30  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-30  |  Report generated 01 Jul 2026, 17:26  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Pathways Quality Award — Excellence (this Area)</t>
+          <t>Clubs Qualifying — Excellence (this Area)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>District Rank</t>
+          <t>Club</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Club</t>
+          <t>Level 1</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Level 1</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
           <t>Level 3</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Ovation 2027</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
           <t>No clubs yet</t>
         </is>
       </c>
+      <c r="B7" s="6" t="inlineStr"/>
       <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1005,13 +987,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1031,84 +1012,70 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Snapshot as of 2026-06-30  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-30  |  Report generated 01 Jul 2026, 17:26  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Pathways Quality Award — Star (this Area)</t>
+          <t>Clubs Qualifying — Star (this Area)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>District Rank</t>
+          <t>Club</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Club</t>
+          <t>Level 1</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Level 1</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
           <t>Level 3</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Commercial Bank Toastmasters Club</t>
         </is>
       </c>
+      <c r="B7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="C7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D7" s="6" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n">
-        <v>23</v>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Lions Toastmasters Club</t>
         </is>
       </c>
+      <c r="B8" s="8" t="n">
+        <v>5</v>
+      </c>
       <c r="C8" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="D8" s="8" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n">
-        <v>41</v>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>The Colombo Toastmasters Club</t>
         </is>
       </c>
+      <c r="B9" s="6" t="n">
+        <v>11</v>
+      </c>
       <c r="C9" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="D9" s="6" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerate reports with rank/disclaimer fixes
</commit_message>
<xml_diff>
--- a/docs/exports/area/Division_A_Area_01.xlsx
+++ b/docs/exports/area/Division_A_Area_01.xlsx
@@ -514,7 +514,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-06-30  |  Report generated 01 Jul 2026, 17:26  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-30  |  Report generated 01 Jul 2026, 17:41  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-06-30  |  Report generated 01 Jul 2026, 17:26  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-30  |  Report generated 01 Jul 2026, 17:41  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-06-30  |  Report generated 01 Jul 2026, 17:26  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-30  |  Report generated 01 Jul 2026, 17:41  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-06-30  |  Report generated 01 Jul 2026, 17:26  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-30  |  Report generated 01 Jul 2026, 17:41  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-06-30  |  Report generated 01 Jul 2026, 17:26  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-30  |  Report generated 01 Jul 2026, 17:41  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix ranking to dense-rank style (1,2,2,3), regenerate reports
</commit_message>
<xml_diff>
--- a/docs/exports/area/Division_A_Area_01.xlsx
+++ b/docs/exports/area/Division_A_Area_01.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Area 01 — Level Totals (Divi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="District-Wide Standing — Ran" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Club Leaderboard (within Are" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Clubs Qualifying — Excellenc" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Clubs Qualifying — Star (thi" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Area 01 — Level Totals (Divi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="District-Wide Standing — Ran" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Club Leaderboard (within Are" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clubs Qualifying — Excellenc" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clubs Qualifying — Star (thi" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -514,7 +514,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-05-24  |  Report generated 02 Jul 2026, 16:21  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-30  |  Report generated 02 Jul 2026, 12:25  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -554,19 +554,19 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D7" s="6" t="n">
         <v>8</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -607,7 +607,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-05-24  |  Report generated 02 Jul 2026, 16:21  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-30  |  Report generated 02 Jul 2026, 12:25  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -653,13 +653,13 @@
         <v>5</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9">
@@ -710,7 +710,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-05-24  |  Report generated 02 Jul 2026, 16:21  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-30  |  Report generated 02 Jul 2026, 12:25  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -773,7 +773,7 @@
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D7" s="6" t="n">
         <v>5</v>
@@ -785,7 +785,7 @@
         <v>2</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H7" s="6" t="n">
         <v>72</v>
@@ -797,26 +797,26 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Lions Toastmasters Club</t>
+          <t>Commercial Bank Toastmasters Club</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E8" s="8" t="n">
         <v>2</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G8" s="8" t="n">
         <v>14</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9">
@@ -825,26 +825,26 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Commercial Bank Toastmasters Club</t>
+          <t>Lions Toastmasters Club</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" s="6" t="n">
         <v>4</v>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>5</v>
       </c>
       <c r="E9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10">
@@ -857,19 +857,19 @@
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D10" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" s="8" t="n">
         <v>2</v>
-      </c>
-      <c r="E10" s="8" t="n">
-        <v>0</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>1</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H10" s="8" t="n">
         <v>20</v>
@@ -939,7 +939,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-05-24  |  Report generated 02 Jul 2026, 16:21  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-30  |  Report generated 02 Jul 2026, 12:25  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-05-24  |  Report generated 02 Jul 2026, 16:21  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-30  |  Report generated 02 Jul 2026, 12:25  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix tiebreaker logic on Total Levels leaderboard, reformat banner as numbered list
</commit_message>
<xml_diff>
--- a/docs/exports/area/Division_A_Area_01.xlsx
+++ b/docs/exports/area/Division_A_Area_01.xlsx
@@ -514,7 +514,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-06-30  |  Report generated 02 Jul 2026, 12:25  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-30  |  Report generated 02 Jul 2026, 12:37  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-06-30  |  Report generated 02 Jul 2026, 12:25  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-30  |  Report generated 02 Jul 2026, 12:37  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-06-30  |  Report generated 02 Jul 2026, 12:25  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-30  |  Report generated 02 Jul 2026, 12:37  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-06-30  |  Report generated 02 Jul 2026, 12:25  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-30  |  Report generated 02 Jul 2026, 12:37  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-06-30  |  Report generated 02 Jul 2026, 12:25  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-30  |  Report generated 02 Jul 2026, 12:37  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct dashboard data to 30 May 2026 snapshot, backfill history
</commit_message>
<xml_diff>
--- a/docs/exports/area/Division_A_Area_01.xlsx
+++ b/docs/exports/area/Division_A_Area_01.xlsx
@@ -514,7 +514,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-05-09  |  Report generated 02 Jul 2026, 18:38  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-05  |  Report generated 02 Jul 2026, 18:44  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -557,7 +557,7 @@
         <v>21</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>6</v>
@@ -566,7 +566,7 @@
         <v>8</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -607,7 +607,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-05-09  |  Report generated 02 Jul 2026, 18:38  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-05  |  Report generated 02 Jul 2026, 18:44  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -650,13 +650,13 @@
         <v>9</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E7" s="6" t="n">
         <v>11</v>
@@ -710,7 +710,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-05-09  |  Report generated 02 Jul 2026, 18:38  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-05  |  Report generated 02 Jul 2026, 18:44  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
         <v>19</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="8">
@@ -816,7 +816,7 @@
         <v>14</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9">
@@ -844,7 +844,7 @@
         <v>13</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10">
@@ -860,7 +860,7 @@
         <v>1</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E10" s="8" t="n">
         <v>0</v>
@@ -869,10 +869,10 @@
         <v>1</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H10" s="8" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11">
@@ -939,7 +939,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-05-09  |  Report generated 02 Jul 2026, 18:38  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-05  |  Report generated 02 Jul 2026, 18:44  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-05-09  |  Report generated 02 Jul 2026, 18:38  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-05  |  Report generated 02 Jul 2026, 18:44  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
31 december 25 update
</commit_message>
<xml_diff>
--- a/docs/exports/area/Division_A_Area_01.xlsx
+++ b/docs/exports/area/Division_A_Area_01.xlsx
@@ -514,14 +514,14 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-06-05  |  Report generated 02 Jul 2026, 18:44  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2025-12-31  |  Report generated 02 Jul 2026, 18:51  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Area 01 — Level Totals (Division Rank #2 of 4)</t>
+          <t>Area 01 — Level Totals (Division Rank #3 of 4)</t>
         </is>
       </c>
     </row>
@@ -554,19 +554,19 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>51</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -607,7 +607,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-06-05  |  Report generated 02 Jul 2026, 18:44  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2025-12-31  |  Report generated 02 Jul 2026, 18:51  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -647,19 +647,19 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>19</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9">
@@ -710,7 +710,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-06-05  |  Report generated 02 Jul 2026, 18:44  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2025-12-31  |  Report generated 02 Jul 2026, 18:51  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -773,19 +773,19 @@
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="H7" s="6" t="n">
         <v>72</v>
@@ -797,26 +797,26 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Lions Toastmasters Club</t>
+          <t>Commercial Bank Toastmasters Club</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D8" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="E8" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="F8" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="G8" s="8" t="n">
-        <v>14</v>
-      </c>
       <c r="H8" s="8" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9">
@@ -825,26 +825,26 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Commercial Bank Toastmasters Club</t>
+          <t>Lions Toastmasters Club</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>31</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10">
@@ -860,7 +860,7 @@
         <v>1</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E10" s="8" t="n">
         <v>0</v>
@@ -869,10 +869,10 @@
         <v>1</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H10" s="8" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11">
@@ -885,7 +885,7 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D11" s="6" t="n">
         <v>0</v>
@@ -897,10 +897,10 @@
         <v>0</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -939,7 +939,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-06-05  |  Report generated 02 Jul 2026, 18:44  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2025-12-31  |  Report generated 02 Jul 2026, 18:51  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-06-05  |  Report generated 02 Jul 2026, 18:44  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2025-12-31  |  Report generated 02 Jul 2026, 18:51  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix award tab computing wrong date's snapshot
</commit_message>
<xml_diff>
--- a/docs/exports/area/Division_A_Area_01.xlsx
+++ b/docs/exports/area/Division_A_Area_01.xlsx
@@ -514,7 +514,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2025-12-31  |  Report generated 02 Jul 2026, 19:02  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2025-12-31  |  Report generated 02 Jul 2026, 19:27  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2025-12-31  |  Report generated 02 Jul 2026, 19:02  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2025-12-31  |  Report generated 02 Jul 2026, 19:27  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2025-12-31  |  Report generated 02 Jul 2026, 19:02  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2025-12-31  |  Report generated 02 Jul 2026, 19:27  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2025-12-31  |  Report generated 02 Jul 2026, 19:02  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2025-12-31  |  Report generated 02 Jul 2026, 19:27  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -987,10 +987,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
   </cols>
@@ -1012,7 +1012,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2025-12-31  |  Report generated 02 Jul 2026, 19:02  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2025-12-31  |  Report generated 02 Jul 2026, 19:27  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -1043,41 +1043,11 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Commercial Bank Toastmasters Club</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Lions Toastmasters Club</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="C8" s="8" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>The Colombo Toastmasters Club</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>2</v>
-      </c>
+          <t>No clubs yet</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr"/>
+      <c r="C7" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
april 30th update test
</commit_message>
<xml_diff>
--- a/docs/exports/area/Division_A_Area_01.xlsx
+++ b/docs/exports/area/Division_A_Area_01.xlsx
@@ -514,7 +514,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2025-10-31  |  Report generated 02 Jul 2026, 19:37  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-04-30  |  Report generated 02 Jul 2026, 19:50  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -554,19 +554,19 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>9</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -607,7 +607,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2025-10-31  |  Report generated 02 Jul 2026, 19:37  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-04-30  |  Report generated 02 Jul 2026, 19:50  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -647,19 +647,19 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9">
@@ -710,7 +710,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2025-10-31  |  Report generated 02 Jul 2026, 19:37  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-04-30  |  Report generated 02 Jul 2026, 19:50  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -769,26 +769,26 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Lions Toastmasters Club</t>
+          <t>The Colombo Toastmasters Club</t>
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>16</v>
+        <v>68</v>
       </c>
     </row>
     <row r="8">
@@ -797,26 +797,26 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>The Colombo Toastmasters Club</t>
+          <t>Lions Toastmasters Club</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="E8" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="D8" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="8" t="n">
-        <v>1</v>
-      </c>
       <c r="F8" s="8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>70</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9">
@@ -825,26 +825,26 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>CEB Toastmasters Club</t>
+          <t>Commercial Bank Toastmasters Club</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>11</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10">
@@ -853,26 +853,26 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Commercial Bank Toastmasters Club</t>
+          <t>CEB Toastmasters Club</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="8" t="n">
         <v>0</v>
-      </c>
-      <c r="D10" s="8" t="n">
-        <v>1</v>
       </c>
       <c r="E10" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H10" s="8" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
@@ -885,7 +885,7 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D11" s="6" t="n">
         <v>0</v>
@@ -897,10 +897,10 @@
         <v>0</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>31</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -939,7 +939,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2025-10-31  |  Report generated 02 Jul 2026, 19:37  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-04-30  |  Report generated 02 Jul 2026, 19:50  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -987,10 +987,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
   </cols>
@@ -1012,7 +1012,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2025-10-31  |  Report generated 02 Jul 2026, 19:37  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-04-30  |  Report generated 02 Jul 2026, 19:50  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -1043,11 +1043,41 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>No clubs yet</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr"/>
+          <t>Commercial Bank Toastmasters Club</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Lions Toastmasters Club</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>The Colombo Toastmasters Club</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update dashboard: April 30 test
</commit_message>
<xml_diff>
--- a/docs/exports/area/Division_A_Area_01.xlsx
+++ b/docs/exports/area/Division_A_Area_01.xlsx
@@ -514,7 +514,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-04-30  |  Report generated 02 Jul 2026, 19:50  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-04-30  |  Report generated 02 Jul 2026, 20:06  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-04-30  |  Report generated 02 Jul 2026, 19:50  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-04-30  |  Report generated 02 Jul 2026, 20:06  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-04-30  |  Report generated 02 Jul 2026, 19:50  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-04-30  |  Report generated 02 Jul 2026, 20:06  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-04-30  |  Report generated 02 Jul 2026, 19:50  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-04-30  |  Report generated 02 Jul 2026, 20:06  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-04-30  |  Report generated 02 Jul 2026, 19:50  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-04-30  |  Report generated 02 Jul 2026, 20:06  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
April 5th Update Data
</commit_message>
<xml_diff>
--- a/docs/exports/area/Division_A_Area_01.xlsx
+++ b/docs/exports/area/Division_A_Area_01.xlsx
@@ -514,7 +514,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-04-30  |  Report generated 02 Jul 2026, 20:06  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-03-05  |  Report generated 02 Jul 2026, 20:33  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -554,19 +554,19 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="C7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="D7" s="6" t="n">
-        <v>8</v>
-      </c>
       <c r="E7" s="6" t="n">
-        <v>48</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -607,7 +607,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-04-30  |  Report generated 02 Jul 2026, 20:06  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-03-05  |  Report generated 02 Jul 2026, 20:33  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -647,19 +647,19 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9">
@@ -710,7 +710,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-04-30  |  Report generated 02 Jul 2026, 20:06  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-03-05  |  Report generated 02 Jul 2026, 20:33  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -779,16 +779,16 @@
         <v>5</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="8">
@@ -801,22 +801,22 @@
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>3</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9">
@@ -829,22 +829,22 @@
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10">
@@ -872,7 +872,7 @@
         <v>2</v>
       </c>
       <c r="H10" s="8" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11">
@@ -885,7 +885,7 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D11" s="6" t="n">
         <v>0</v>
@@ -897,10 +897,10 @@
         <v>0</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -939,7 +939,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-04-30  |  Report generated 02 Jul 2026, 20:06  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-03-05  |  Report generated 02 Jul 2026, 20:33  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -987,10 +987,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
   </cols>
@@ -1012,7 +1012,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-04-30  |  Report generated 02 Jul 2026, 20:06  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-03-05  |  Report generated 02 Jul 2026, 20:33  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -1043,41 +1043,11 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Commercial Bank Toastmasters Club</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Lions Toastmasters Club</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="C8" s="8" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>The Colombo Toastmasters Club</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>2</v>
-      </c>
+          <t>No clubs yet</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr"/>
+      <c r="C7" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Optimize dashboard layout for smartphone screens
Division/area tables were forcing horizontal scroll on phones that hid
key numbers (like area totals) off-screen. Drop decorative
composition/club-count columns on mobile, let tables auto-fit instead
of forcing a min-width, restructure the division accordion header and
club leaderboard rows to wrap/stack instead of squeezing into fixed
grid columns, and tighten spacing/type sizes for small viewports.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/exports/area/Division_A_Area_01.xlsx
+++ b/docs/exports/area/Division_A_Area_01.xlsx
@@ -514,7 +514,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-06-30  |  Report generated 04 Jul 2026, 13:03  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-30  |  Report generated 04 Jul 2026, 13:24  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-06-30  |  Report generated 04 Jul 2026, 13:03  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-30  |  Report generated 04 Jul 2026, 13:24  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-06-30  |  Report generated 04 Jul 2026, 13:03  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-30  |  Report generated 04 Jul 2026, 13:24  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-06-30  |  Report generated 04 Jul 2026, 13:03  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-30  |  Report generated 04 Jul 2026, 13:24  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-06-30  |  Report generated 04 Jul 2026, 13:03  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-06-30  |  Report generated 04 Jul 2026, 13:24  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>

</xml_diff>